<commit_message>
Add the possibility to specify who places the order
</commit_message>
<xml_diff>
--- a/assets/order_model_example.xlsx
+++ b/assets/order_model_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://abb-my.sharepoint.com/personal/baptiste_michot_be_abb_com/Documents/Documents/Imprimantes/PrintersABB/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="11_17A98B1BBDF679A1B9F056B7BF0A2FB473B653D6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57DA6BD9-690E-4346-9BC5-48A190923E51}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_17A98B1BBDF679A1B9F056B7BF0A2FB473B653D6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2880842B-539D-4B06-A8BA-3FC3FFF6E697}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="297" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,12 +141,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="6">
+    <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="#,##0.00\ &quot;€&quot;"/>
-    <numFmt numFmtId="166" formatCode="_ [$€-413]\ * #,##0.00_ ;_ [$€-413]\ * \-#,##0.00_ ;_ [$€-413]\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="167" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
     <numFmt numFmtId="168" formatCode="[$EUR]\ #,##0.00_);[Red]\([$EUR]\ #,##0.00\)"/>
     <numFmt numFmtId="169" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
   </numFmts>
@@ -464,7 +463,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="169" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
@@ -472,8 +471,9 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="43" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="22" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -614,19 +614,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -641,17 +629,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -663,9 +642,6 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -687,9 +663,27 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Comma" xfId="3" builtinId="3"/>
+    <cellStyle name="Currency" xfId="4" builtinId="4"/>
     <cellStyle name="Euro" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1073,7 +1067,7 @@
     <col min="7" max="7" width="26.88671875" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="10.5546875" customWidth="1"/>
-    <col min="10" max="10" width="21" customWidth="1"/>
+    <col min="10" max="10" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -1090,9 +1084,9 @@
         <v>31</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="76"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="76"/>
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+      <c r="J3" s="72"/>
     </row>
     <row r="4" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="49" t="s">
@@ -1101,71 +1095,71 @@
       <c r="G4" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="85"/>
-      <c r="I4" s="86"/>
-      <c r="J4" s="87"/>
+      <c r="H4" s="78"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="80"/>
     </row>
     <row r="5" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="49"/>
       <c r="G5" s="51"/>
-      <c r="H5" s="82"/>
-      <c r="I5" s="78"/>
-      <c r="J5" s="79"/>
+      <c r="H5" s="77"/>
+      <c r="I5" s="74"/>
+      <c r="J5" s="75"/>
     </row>
     <row r="6" spans="1:10" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="50"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="78"/>
-      <c r="J6" s="79"/>
+      <c r="H6" s="77"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="75"/>
     </row>
     <row r="7" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="82"/>
-      <c r="I7" s="78"/>
-      <c r="J7" s="79"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="75"/>
     </row>
     <row r="8" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="82"/>
-      <c r="I8" s="78"/>
-      <c r="J8" s="79"/>
+      <c r="H8" s="77"/>
+      <c r="I8" s="74"/>
+      <c r="J8" s="75"/>
     </row>
     <row r="9" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="82"/>
-      <c r="I9" s="78"/>
-      <c r="J9" s="79"/>
+      <c r="H9" s="77"/>
+      <c r="I9" s="74"/>
+      <c r="J9" s="75"/>
     </row>
     <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="49"/>
-      <c r="H10" s="82"/>
-      <c r="I10" s="78"/>
-      <c r="J10" s="79"/>
+      <c r="H10" s="77"/>
+      <c r="I10" s="74"/>
+      <c r="J10" s="75"/>
     </row>
     <row r="11" spans="1:10" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49"/>
-      <c r="H11" s="82"/>
-      <c r="I11" s="78"/>
-      <c r="J11" s="79"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="74"/>
+      <c r="J11" s="75"/>
     </row>
     <row r="12" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="80" t="s">
+      <c r="C12" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="78"/>
-      <c r="H12" s="93"/>
-      <c r="I12" s="76"/>
-      <c r="J12" s="92"/>
+      <c r="D12" s="74"/>
+      <c r="H12" s="85"/>
+      <c r="I12" s="72"/>
+      <c r="J12" s="84"/>
     </row>
     <row r="13" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
@@ -1179,11 +1173,11 @@
         <v>3</v>
       </c>
       <c r="B15" s="5"/>
-      <c r="C15" s="98">
+      <c r="C15" s="90">
         <f ca="1">TODAY()</f>
-        <v>46105</v>
-      </c>
-      <c r="D15" s="99"/>
+        <v>46107</v>
+      </c>
+      <c r="D15" s="91"/>
     </row>
     <row r="16" spans="1:10" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="2"/>
@@ -1250,180 +1244,180 @@
       <c r="F22" s="68"/>
       <c r="G22" s="68"/>
       <c r="H22" s="66"/>
-      <c r="I22" s="94"/>
-      <c r="J22" s="87"/>
+      <c r="I22" s="86"/>
+      <c r="J22" s="80"/>
     </row>
     <row r="23" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="69">
         <v>1</v>
       </c>
-      <c r="B23" s="100" t="s">
+      <c r="B23" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="78"/>
-      <c r="D23" s="78"/>
-      <c r="E23" s="78"/>
-      <c r="F23" s="78"/>
-      <c r="G23" s="79"/>
-      <c r="H23" s="70">
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="75"/>
+      <c r="H23" s="93">
         <v>238.3</v>
       </c>
-      <c r="I23" s="83">
+      <c r="I23" s="94">
         <f t="shared" ref="I23:I31" si="0">IF(H23="","",H23*A23)</f>
         <v>238.3</v>
       </c>
-      <c r="J23" s="79"/>
+      <c r="J23" s="95"/>
     </row>
     <row r="24" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="69">
         <v>1</v>
       </c>
-      <c r="B24" s="77" t="s">
+      <c r="B24" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="78"/>
-      <c r="D24" s="78"/>
-      <c r="E24" s="78"/>
-      <c r="F24" s="78"/>
-      <c r="G24" s="79"/>
-      <c r="H24" s="71">
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="96">
         <v>234.65</v>
       </c>
-      <c r="I24" s="81">
+      <c r="I24" s="94">
         <f t="shared" si="0"/>
         <v>234.65</v>
       </c>
-      <c r="J24" s="79"/>
+      <c r="J24" s="95"/>
     </row>
     <row r="25" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="72">
+      <c r="A25" s="70">
         <v>4</v>
       </c>
-      <c r="B25" s="77" t="s">
+      <c r="B25" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="C25" s="78"/>
-      <c r="D25" s="78"/>
-      <c r="E25" s="78"/>
-      <c r="F25" s="78"/>
-      <c r="G25" s="79"/>
-      <c r="H25" s="70">
+      <c r="C25" s="74"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="74"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="93">
         <v>233.9</v>
       </c>
-      <c r="I25" s="81">
+      <c r="I25" s="94">
         <f t="shared" si="0"/>
         <v>935.6</v>
       </c>
-      <c r="J25" s="79"/>
+      <c r="J25" s="95"/>
     </row>
     <row r="26" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="72">
+      <c r="A26" s="70">
         <v>1</v>
       </c>
-      <c r="B26" s="77" t="s">
+      <c r="B26" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="78"/>
-      <c r="D26" s="78"/>
-      <c r="E26" s="78"/>
-      <c r="F26" s="78"/>
-      <c r="G26" s="79"/>
-      <c r="H26" s="70">
+      <c r="C26" s="74"/>
+      <c r="D26" s="74"/>
+      <c r="E26" s="74"/>
+      <c r="F26" s="74"/>
+      <c r="G26" s="75"/>
+      <c r="H26" s="93">
         <v>217.37</v>
       </c>
-      <c r="I26" s="81">
+      <c r="I26" s="94">
         <f t="shared" si="0"/>
         <v>217.37</v>
       </c>
-      <c r="J26" s="79"/>
+      <c r="J26" s="95"/>
     </row>
     <row r="27" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="72"/>
-      <c r="B27" s="77"/>
-      <c r="C27" s="78"/>
-      <c r="D27" s="78"/>
-      <c r="E27" s="78"/>
-      <c r="F27" s="78"/>
-      <c r="G27" s="79"/>
-      <c r="H27" s="73"/>
-      <c r="I27" s="84" t="str">
+      <c r="A27" s="70"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="74"/>
+      <c r="D27" s="74"/>
+      <c r="E27" s="74"/>
+      <c r="F27" s="74"/>
+      <c r="G27" s="75"/>
+      <c r="H27" s="93"/>
+      <c r="I27" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J27" s="79"/>
+      <c r="J27" s="95"/>
     </row>
     <row r="28" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="72"/>
-      <c r="B28" s="77"/>
-      <c r="C28" s="78"/>
-      <c r="D28" s="78"/>
-      <c r="E28" s="78"/>
-      <c r="F28" s="78"/>
-      <c r="G28" s="79"/>
-      <c r="H28" s="74"/>
-      <c r="I28" s="84" t="str">
+      <c r="A28" s="70"/>
+      <c r="B28" s="73"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="74"/>
+      <c r="G28" s="75"/>
+      <c r="H28" s="93"/>
+      <c r="I28" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J28" s="79"/>
+      <c r="J28" s="95"/>
     </row>
     <row r="29" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="72"/>
-      <c r="B29" s="77"/>
-      <c r="C29" s="78"/>
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
-      <c r="F29" s="78"/>
-      <c r="G29" s="79"/>
-      <c r="H29" s="72"/>
-      <c r="I29" s="84" t="str">
+      <c r="A29" s="70"/>
+      <c r="B29" s="73"/>
+      <c r="C29" s="74"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="74"/>
+      <c r="F29" s="74"/>
+      <c r="G29" s="75"/>
+      <c r="H29" s="93"/>
+      <c r="I29" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J29" s="79"/>
+      <c r="J29" s="95"/>
       <c r="M29" s="63"/>
     </row>
     <row r="30" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="72"/>
-      <c r="B30" s="77"/>
-      <c r="C30" s="78"/>
-      <c r="D30" s="78"/>
-      <c r="E30" s="78"/>
-      <c r="F30" s="78"/>
-      <c r="G30" s="79"/>
-      <c r="H30" s="72"/>
-      <c r="I30" s="84" t="str">
+      <c r="A30" s="70"/>
+      <c r="B30" s="73"/>
+      <c r="C30" s="74"/>
+      <c r="D30" s="74"/>
+      <c r="E30" s="74"/>
+      <c r="F30" s="74"/>
+      <c r="G30" s="75"/>
+      <c r="H30" s="93"/>
+      <c r="I30" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J30" s="79"/>
+      <c r="J30" s="95"/>
     </row>
     <row r="31" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="72"/>
-      <c r="B31" s="77"/>
-      <c r="C31" s="78"/>
-      <c r="D31" s="78"/>
-      <c r="E31" s="78"/>
-      <c r="F31" s="78"/>
-      <c r="G31" s="79"/>
-      <c r="H31" s="72"/>
-      <c r="I31" s="84" t="str">
+      <c r="A31" s="70"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="74"/>
+      <c r="D31" s="74"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="74"/>
+      <c r="G31" s="75"/>
+      <c r="H31" s="93"/>
+      <c r="I31" s="94" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J31" s="79"/>
+      <c r="J31" s="95"/>
     </row>
     <row r="32" spans="1:13" ht="29.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="75"/>
+      <c r="A32" s="71"/>
       <c r="B32" s="65"/>
       <c r="C32" s="65"/>
       <c r="D32" s="65"/>
       <c r="E32" s="65"/>
       <c r="F32" s="65"/>
       <c r="G32" s="65"/>
-      <c r="H32" s="75"/>
-      <c r="I32" s="91"/>
-      <c r="J32" s="92"/>
+      <c r="H32" s="97"/>
+      <c r="I32" s="98"/>
+      <c r="J32" s="99"/>
     </row>
     <row r="33" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
@@ -1431,11 +1425,11 @@
       <c r="H33" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="I33" s="95">
+      <c r="I33" s="87">
         <f>SUM(I23:J32)</f>
         <v>1625.92</v>
       </c>
-      <c r="J33" s="79"/>
+      <c r="J33" s="75"/>
     </row>
     <row r="34" spans="1:10" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17"/>
@@ -1453,10 +1447,10 @@
       <c r="A35" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B35" s="90"/>
-      <c r="C35" s="89"/>
-      <c r="D35" s="89"/>
-      <c r="E35" s="79"/>
+      <c r="B35" s="83"/>
+      <c r="C35" s="82"/>
+      <c r="D35" s="82"/>
+      <c r="E35" s="75"/>
       <c r="F35" s="56" t="s">
         <v>13</v>
       </c>
@@ -1479,24 +1473,24 @@
       <c r="A37" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="97"/>
-      <c r="C37" s="89"/>
-      <c r="D37" s="89"/>
-      <c r="E37" s="89"/>
+      <c r="B37" s="89"/>
+      <c r="C37" s="82"/>
+      <c r="D37" s="82"/>
+      <c r="E37" s="82"/>
       <c r="F37" s="59" t="s">
         <v>15</v>
       </c>
       <c r="G37" s="54"/>
-      <c r="H37" s="96"/>
-      <c r="I37" s="89"/>
+      <c r="H37" s="88"/>
+      <c r="I37" s="82"/>
       <c r="J37" s="44"/>
     </row>
     <row r="38" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="24"/>
-      <c r="B38" s="88"/>
-      <c r="C38" s="89"/>
-      <c r="D38" s="89"/>
-      <c r="E38" s="89"/>
+      <c r="B38" s="81"/>
+      <c r="C38" s="82"/>
+      <c r="D38" s="82"/>
+      <c r="E38" s="82"/>
       <c r="F38" s="61"/>
       <c r="G38" s="52"/>
       <c r="H38" s="53"/>
@@ -1519,10 +1513,10 @@
       <c r="A40" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="97"/>
-      <c r="C40" s="89"/>
-      <c r="D40" s="89"/>
-      <c r="E40" s="89"/>
+      <c r="B40" s="89"/>
+      <c r="C40" s="82"/>
+      <c r="D40" s="82"/>
+      <c r="E40" s="82"/>
       <c r="F40" s="62"/>
       <c r="G40" s="52"/>
       <c r="H40" s="53"/>
@@ -1531,10 +1525,10 @@
     </row>
     <row r="41" spans="1:10" s="3" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24"/>
-      <c r="B41" s="88"/>
-      <c r="C41" s="89"/>
-      <c r="D41" s="89"/>
-      <c r="E41" s="89"/>
+      <c r="B41" s="81"/>
+      <c r="C41" s="82"/>
+      <c r="D41" s="82"/>
+      <c r="E41" s="82"/>
       <c r="F41" s="62"/>
       <c r="G41" s="52"/>
       <c r="H41" s="53"/>

</xml_diff>